<commit_message>
Update Excel evidence files; remove temp files
Add FinalReport/Evidence/irish_model_summary_charts.xlsx, update FinalReport/Evidence/wav2vec_vs_mfcc.xlsx and FinalReport/Evidence/wav2vec_vs_mfcc/irish_model_summary_charts.xlsx with refreshed chart/metric data for the final report, and remove MS Office temporary files (~$irish_model_summary_charts.xlsx and ~$wav2vec_vs_mfcc.xlsx).
</commit_message>
<xml_diff>
--- a/FinalReport/Evidence/wav2vec_vs_mfcc/irish_model_summary_charts.xlsx
+++ b/FinalReport/Evidence/wav2vec_vs_mfcc/irish_model_summary_charts.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cianan/Documents/College/GitHub/FYP/Experiments/AutoModels/results/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cianan/Documents/College/GitHub/FYP/FinalReport/Evidence/wav2vec_vs_mfcc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33809487-A0D8-B04D-BA23-BE4EB0BE3B69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D20F56B-E86A-574E-9194-3102573DC3E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38400" yWindow="1360" windowWidth="38400" windowHeight="21800" firstSheet="4" activeTab="10" xr2:uid="{4FF49A69-2F49-B14A-A75D-0C6888D117A2}"/>
+    <workbookView xWindow="38400" yWindow="1360" windowWidth="38400" windowHeight="21800" firstSheet="4" activeTab="8" xr2:uid="{4FF49A69-2F49-B14A-A75D-0C6888D117A2}"/>
   </bookViews>
   <sheets>
     <sheet name="irish_model_summary_rebuilt" sheetId="1" r:id="rId1"/>
@@ -4721,6 +4721,545 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:sysClr>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Irish Dataset:  </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-IE" sz="1400" b="1" i="0" u="none" strike="noStrike" baseline="0"/>
+              <a:t>Average Improvement Over Random Baseline by Model</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" b="1"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Chart4 - relativeAccuracyModel'!$H$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>avg_relative_improvement</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="bg1"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="inEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Chart4 - relativeAccuracyModel'!$G$2:$G$12</c:f>
+              <c:strCache>
+                <c:ptCount val="11"/>
+                <c:pt idx="0">
+                  <c:v>k-NN (k=1)</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>k-NN (k=3)</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>k-NN (k=5)</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>k-NN (k=7)</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>k-NN (k=11)</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>SVM (RBF Kernel)</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Random Forest</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Naive Bayes</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Logistic Regression</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>SVM (Linear)</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Logistic Regression (Weighted)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Chart4 - relativeAccuracyModel'!$H$2:$H$12</c:f>
+              <c:numCache>
+                <c:formatCode>0.00%</c:formatCode>
+                <c:ptCount val="11"/>
+                <c:pt idx="0">
+                  <c:v>0.22058773318991201</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.24318918448075769</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.24736137814645034</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.26890001186548718</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.27021457756549483</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.29743821886594501</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.31737390451873354</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.33499851349043003</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.36592986953842538</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.37003461658216513</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.40344671029958601</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-C22D-0C45-8A27-A1330C89E94E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="84"/>
+        <c:overlap val="-27"/>
+        <c:axId val="435735456"/>
+        <c:axId val="435670448"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="435735456"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-GB" sz="1200"/>
+                  <a:t>Model</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="435670448"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="435670448"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-IE" sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0"/>
+                  <a:t>Relative Improvement </a:t>
+                </a:r>
+                <a:endParaRPr lang="en-GB" sz="1200"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-GB"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0.00%" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="435735456"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
@@ -7576,6 +8115,473 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
+              <a:rPr lang="en-US" b="1"/>
+              <a:t>Irish</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" b="1" baseline="0"/>
+              <a:t> Dataset: </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" b="1"/>
+              <a:t>Best Model Per Task</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Chart 2 - BestModelPerTask'!$G$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>balanced_accuracy_mean</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="0070C0"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Chart 2 - BestModelPerTask'!$F$2:$F$7</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>Dáil Speakers
+Logistic Regression</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Four Provinces
+SVM (Linear)</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Ulster, Leinster, and Rest
+SVM (RBF Kernel)</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Leinster vs Rest
+Logistic Regression (Weighted)</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Ulster vs Rest
+Logistic Regression (Weighted)</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Dáil vs Northern Ireland
+Naive Bayes</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Chart 2 - BestModelPerTask'!$G$2:$G$7</c:f>
+              <c:numCache>
+                <c:formatCode>0.00%</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>0.27210886725816702</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.39387690904640299</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.52408969936051997</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.61580000000000001</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.74775796701111596</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.78742267907035202</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-FC17-C142-8CB0-BC342651D6BF}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="50"/>
+        <c:axId val="1389255183"/>
+        <c:axId val="1389054559"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1389255183"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-GB" sz="1200" b="1"/>
+                  <a:t>Task</a:t>
+                </a:r>
+              </a:p>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1200" b="1"/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-GB" sz="1200" b="1"/>
+                  <a:t>------</a:t>
+                </a:r>
+                <a:br>
+                  <a:rPr lang="en-GB" sz="1200" b="1"/>
+                </a:br>
+                <a:r>
+                  <a:rPr lang="en-GB" sz="1200" b="1"/>
+                  <a:t>Model</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1389054559"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1389054559"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-GB" sz="1200" b="1"/>
+                  <a:t>Balanced Accuracy</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-GB" sz="1200" b="1" baseline="0"/>
+                  <a:t> Mean</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0.00%" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1389255183"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
               <a:rPr lang="en-US" sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
                   <a:sysClr val="windowText" lastClr="000000">
@@ -7923,7 +8929,7 @@
               </a:p>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1200" b="0"/>
+                  <a:defRPr sz="1200"/>
                 </a:pPr>
                 <a:endParaRPr lang="en-GB" sz="1200" b="0" i="0"/>
               </a:p>
@@ -8045,546 +9051,47 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-GB"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US" sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-                <a:solidFill>
-                  <a:sysClr val="windowText" lastClr="000000">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:sysClr>
-                </a:solidFill>
-              </a:rPr>
-              <a:t>Irish Dataset:  </a:t>
-            </a:r>
-            <a:r>
-              <a:rPr lang="en-IE" sz="1400" b="1" i="0" u="none" strike="noStrike" baseline="0"/>
-              <a:t>Average Improvement Over Random Baseline by Model</a:t>
-            </a:r>
-            <a:endParaRPr lang="en-US" b="1"/>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout/>
-      <c:barChart>
-        <c:barDir val="col"/>
-        <c:grouping val="clustered"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>'Chart4 - relativeAccuracyModel'!$H$1</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>avg_relative_improvement</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent1"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:dLbls>
-            <c:spPr>
-              <a:noFill/>
-              <a:ln>
-                <a:noFill/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-                <a:spAutoFit/>
-              </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="bg1"/>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:endParaRPr lang="en-US"/>
-              </a:p>
-            </c:txPr>
-            <c:dLblPos val="inEnd"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="1"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showBubbleSize val="0"/>
-            <c:showLeaderLines val="0"/>
-            <c:extLst>
-              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:showLeaderLines val="1"/>
-                <c15:leaderLines>
-                  <c:spPr>
-                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="35000"/>
-                          <a:lumOff val="65000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                      <a:round/>
-                    </a:ln>
-                    <a:effectLst/>
-                  </c:spPr>
-                </c15:leaderLines>
-              </c:ext>
-            </c:extLst>
-          </c:dLbls>
-          <c:cat>
-            <c:strRef>
-              <c:f>'Chart4 - relativeAccuracyModel'!$G$2:$G$12</c:f>
-              <c:strCache>
-                <c:ptCount val="11"/>
-                <c:pt idx="0">
-                  <c:v>k-NN (k=1)</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>k-NN (k=3)</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>k-NN (k=5)</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>k-NN (k=7)</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>k-NN (k=11)</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>SVM (RBF Kernel)</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>Random Forest</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>Naive Bayes</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>Logistic Regression</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>SVM (Linear)</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>Logistic Regression (Weighted)</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'Chart4 - relativeAccuracyModel'!$H$2:$H$12</c:f>
-              <c:numCache>
-                <c:formatCode>0.00%</c:formatCode>
-                <c:ptCount val="11"/>
-                <c:pt idx="0">
-                  <c:v>0.22058773318991201</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.24318918448075769</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.24736137814645034</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0.26890001186548718</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0.27021457756549483</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0.29743821886594501</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>0.31737390451873354</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>0.33499851349043003</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>0.36592986953842538</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>0.37003461658216513</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>0.40344671029958601</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-C22D-0C45-8A27-A1330C89E94E}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:gapWidth val="84"/>
-        <c:overlap val="-27"/>
-        <c:axId val="435735456"/>
-        <c:axId val="435670448"/>
-      </c:barChart>
-      <c:catAx>
-        <c:axId val="435735456"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="65000"/>
-                        <a:lumOff val="35000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr lang="en-GB" sz="1200"/>
-                  <a:t>Model</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:overlay val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
-        </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="15000"/>
-                <a:lumOff val="85000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="435670448"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="435670448"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="65000"/>
-                        <a:lumOff val="35000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr lang="en-IE" sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0"/>
-                  <a:t>Relative Improvement </a:t>
-                </a:r>
-                <a:endParaRPr lang="en-GB" sz="1200"/>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:overlay val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-GB"/>
-            </a:p>
-          </c:txPr>
-        </c:title>
-        <c:numFmt formatCode="0.00%" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="435735456"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="en-US"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
 </file>
 
-<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/colors10.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -9449,8 +9956,8 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="216">
+<file path=xl/charts/style10.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
@@ -9654,6 +10161,509 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="216">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
@@ -12480,7 +13490,7 @@
 </file>
 
 <file path=xl/charts/style8.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="297">
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="216">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
@@ -12985,7 +13995,7 @@
 </file>
 
 <file path=xl/charts/style9.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="297">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
@@ -13189,22 +14199,23 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
         <a:schemeClr val="dk1">
-          <a:lumMod val="65000"/>
-          <a:lumOff val="35000"/>
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
         </a:schemeClr>
       </a:solidFill>
-      <a:ln w="9525">
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
             <a:lumMod val="65000"/>
             <a:lumOff val="35000"/>
           </a:schemeClr>
         </a:solidFill>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:downBar>
@@ -13309,8 +14320,8 @@
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
-            <a:lumMod val="75000"/>
-            <a:lumOff val="25000"/>
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -13442,19 +14453,20 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
         <a:schemeClr val="lt1"/>
       </a:solidFill>
-      <a:ln w="9525">
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
           </a:schemeClr>
         </a:solidFill>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:upBar>
@@ -13776,6 +14788,44 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>1397000</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>138546</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>628842</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>125845</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00AEE2B3-11AE-0843-A7B7-15448F7EC3D7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>

</xml_diff>